<commit_message>
- Fleet VT v6 (KiNESYS_CEA, n0.4, high) - RE SubRES with 2712 VRE clusters - Conv tech VT V6 + IEA2025 cost scenarios - Timeslice parameters (ts_48)
</commit_message>
<xml_diff>
--- a/SubRes_Tmpl/SubRES_H2-Production.xlsx
+++ b/SubRes_Tmpl/SubRES_H2-Production.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\KiNESYS_BattCircularity-main\SubRes_Tmpl\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CA87521-2B74-460B-A4E2-F505E635EBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="8260" activeTab="5"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SectFuel" sheetId="2" r:id="rId1"/>
@@ -83,12 +89,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Rocco De Miglio</author>
   </authors>
   <commentList>
-    <comment ref="O39" authorId="0">
+    <comment ref="O39" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -116,13 +122,13 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>xli9</author>
     <author>Amit Kanudia</author>
   </authors>
   <commentList>
-    <comment ref="BA16" authorId="0">
+    <comment ref="BA16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000001000000}">
       <text>
         <r>
           <rPr>
@@ -144,7 +150,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y17" authorId="0">
+    <comment ref="Y17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000002000000}">
       <text>
         <r>
           <rPr>
@@ -166,7 +172,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P19" authorId="1">
+    <comment ref="P19" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0500-000003000000}">
       <text>
         <r>
           <rPr>
@@ -190,7 +196,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA19" authorId="0">
+    <comment ref="BA19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000004000000}">
       <text>
         <r>
           <rPr>
@@ -212,7 +218,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA22" authorId="0">
+    <comment ref="BA22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000005000000}">
       <text>
         <r>
           <rPr>
@@ -234,7 +240,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA25" authorId="0">
+    <comment ref="BA25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000006000000}">
       <text>
         <r>
           <rPr>
@@ -256,7 +262,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA28" authorId="0">
+    <comment ref="BA28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000007000000}">
       <text>
         <r>
           <rPr>
@@ -278,7 +284,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="BA31" authorId="0">
+    <comment ref="BA31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000008000000}">
       <text>
         <r>
           <rPr>
@@ -300,7 +306,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C33" authorId="0">
+    <comment ref="C33" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-000009000000}">
       <text>
         <r>
           <rPr>
@@ -322,14 +328,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="AY34" authorId="0">
+    <comment ref="AY34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0500-00000A000000}">
       <text>
         <r>
           <rPr>
             <b/>
             <sz val="9"/>
             <rFont val="Times New Roman"/>
-            <charset val="0"/>
           </rPr>
           <t>xli9:</t>
         </r>
@@ -337,7 +342,6 @@
           <rPr>
             <sz val="9"/>
             <rFont val="Times New Roman"/>
-            <charset val="0"/>
           </rPr>
           <t xml:space="preserve">
 1,000-MW, 10-hour facility — so in US-style capacity-expansion modeling, 10 h is effectively the central assumption for new closed-loop PSH.
@@ -1083,19 +1087,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="9">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="176" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* \-??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;$&quot;* #,##0_-;\-&quot;$&quot;* #,##0_-;_-&quot;$&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="\Te\x\t"/>
-    <numFmt numFmtId="179" formatCode="#,##0.000"/>
-    <numFmt numFmtId="180" formatCode="#,##0.0_ "/>
-    <numFmt numFmtId="181" formatCode="0.0"/>
-    <numFmt numFmtId="182" formatCode="0.000"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="5">
+    <numFmt numFmtId="168" formatCode="\Te\x\t"/>
+    <numFmt numFmtId="169" formatCode="#,##0.000"/>
+    <numFmt numFmtId="170" formatCode="#,##0.0_ "/>
+    <numFmt numFmtId="171" formatCode="0.0"/>
+    <numFmt numFmtId="172" formatCode="0.000"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1123,7 +1123,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.2"/>
+      <sz val="10.199999999999999"/>
       <color rgb="FF212529"/>
       <name val="Segoe UI"/>
       <charset val="134"/>
@@ -1225,130 +1225,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="Times New Roman"/>
-      <charset val="0"/>
     </font>
     <font>
       <b/>
@@ -1376,10 +1254,16 @@
       <b/>
       <sz val="9"/>
       <name val="Times New Roman"/>
-      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="49">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1394,7 +1278,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.349986266670736"/>
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1406,7 +1290,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799951170384838"/>
+        <fgColor theme="4" tint="0.79992065187536243"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1418,7 +1302,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399914548173467"/>
+        <fgColor theme="9" tint="0.39988402966399123"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1430,7 +1314,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.0499893185216834"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1454,7 +1338,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799920651875362"/>
+        <fgColor theme="5" tint="0.79989013336588644"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1472,7 +1356,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799920651875362"/>
+        <fgColor theme="9" tint="0.79989013336588644"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1484,7 +1368,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1500,176 +1384,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="34">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -1811,7 +1527,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.399914548173467"/>
+        <color theme="4" tint="0.39988402966399123"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1857,7 +1573,7 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="0" tint="-0.249946592608417"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </left>
       <right/>
       <top/>
@@ -1867,7 +1583,7 @@
     <border>
       <left/>
       <right style="thin">
-        <color theme="0" tint="-0.249946592608417"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </right>
       <top/>
       <bottom/>
@@ -1884,7 +1600,7 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="0" tint="-0.249946592608417"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </left>
       <right/>
       <top style="thin">
@@ -1896,7 +1612,7 @@
     <border>
       <left/>
       <right style="thin">
-        <color theme="0" tint="-0.249946592608417"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </right>
       <top style="thin">
         <color auto="1"/>
@@ -1937,7 +1653,7 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="0" tint="-0.249946592608417"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </left>
       <right/>
       <top/>
@@ -1949,7 +1665,7 @@
     <border>
       <left/>
       <right style="thin">
-        <color theme="0" tint="-0.249946592608417"/>
+        <color theme="0" tint="-0.24994659260841701"/>
       </right>
       <top/>
       <bottom style="thin">
@@ -1957,283 +1673,65 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="51">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="27" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="9" fontId="24" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="29" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="30" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="29" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="31" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="32" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="33" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="185">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="178" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="179" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="49" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="6" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -2252,12 +1750,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
@@ -2267,7 +1765,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2276,42 +1774,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="50"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="13"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="15"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="14"/>
-    <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="50" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="50" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="50" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="168" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="7"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="2"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="4"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="3"/>
+    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="7" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="7" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="7" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="24" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="5" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2329,19 +1815,16 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="13" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2362,13 +1845,13 @@
     <xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2395,25 +1878,25 @@
     <xf numFmtId="0" fontId="14" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="14" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="14" fillId="13" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="13" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="13" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="14" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="13" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="13" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="13" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2425,25 +1908,25 @@
     <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="14" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="14" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="14" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="14" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="14" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="14" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="14" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2455,25 +1938,25 @@
     <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="15" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="15" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="15" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="15" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="15" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="15" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="15" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="15" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="15" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2485,25 +1968,25 @@
     <xf numFmtId="0" fontId="13" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="16" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="16" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="16" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="16" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="16" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="16" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="16" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2518,25 +2001,25 @@
     <xf numFmtId="0" fontId="13" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="18" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="18" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="18" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="18" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="18" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="18" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="18" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="18" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="18" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="18" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="17" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2548,25 +2031,25 @@
     <xf numFmtId="0" fontId="13" fillId="16" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="16" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="16" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="16" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="14" fillId="16" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="16" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="16" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="16" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="14" fillId="16" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2575,25 +2058,25 @@
     <xf numFmtId="1" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="19" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="19" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="19" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="19" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2605,25 +2088,25 @@
     <xf numFmtId="1" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="20" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="20" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="20" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="20" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="20" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="20" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="20" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="20" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2635,25 +2118,25 @@
     <xf numFmtId="0" fontId="13" fillId="19" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="13" fillId="19" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="19" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="13" fillId="19" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="13" fillId="19" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="19" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="19" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2664,72 +2147,54 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="51">
+  <cellStyles count="8">
+    <cellStyle name="Heading 2" xfId="2" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="3" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="4" builtinId="19"/>
+    <cellStyle name="Neutral" xfId="5" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 10" xfId="49"/>
-    <cellStyle name="Normal 2" xfId="50"/>
+    <cellStyle name="Normal 10" xfId="6" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="Normal 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="New Microsoft Excel Worksheet"/>
       <sheetName val="AGR_Fuels"/>
@@ -2745,8 +2210,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="IEA Data"/>
       <sheetName val="E&amp;D Drivers"/>
@@ -2858,8 +2326,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="IEA Data"/>
       <sheetName val="E&amp;D Drivers"/>
@@ -2971,8 +2442,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Cover"/>
       <sheetName val="H2 transport"/>
@@ -3008,8 +2482,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Cover"/>
       <sheetName val="ELC_Lists"/>
@@ -3043,8 +2520,11 @@
 </file>
 
 <file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Discuss_log"/>
       <sheetName val="Cover"/>
@@ -3089,22 +2569,22 @@
       <sheetData sheetId="13">
         <row r="6">
           <cell r="AW6">
-            <v>0.0473</v>
+            <v>4.7300000000000002E-2</v>
           </cell>
         </row>
         <row r="7">
           <cell r="AW7">
-            <v>0.171166666666667</v>
+            <v>0.17116666666666699</v>
           </cell>
         </row>
         <row r="8">
           <cell r="AW8">
-            <v>0.466366666666667</v>
+            <v>0.46636666666666698</v>
           </cell>
         </row>
         <row r="9">
           <cell r="AW9">
-            <v>0.0956666666666667</v>
+            <v>9.5666666666666705E-2</v>
           </cell>
         </row>
       </sheetData>
@@ -3376,29 +2856,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:P7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="11.8636363636364" customWidth="1"/>
-    <col min="3" max="3" width="9.4" customWidth="1"/>
-    <col min="4" max="4" width="15.2636363636364" customWidth="1"/>
+    <col min="2" max="2" width="11.86328125" customWidth="1"/>
+    <col min="3" max="3" width="9.3984375" customWidth="1"/>
+    <col min="4" max="4" width="15.265625" customWidth="1"/>
     <col min="5" max="5" width="4" customWidth="1"/>
-    <col min="6" max="6" width="6.4" customWidth="1"/>
-    <col min="7" max="7" width="8.26363636363636" customWidth="1"/>
-    <col min="9" max="9" width="11.2636363636364" customWidth="1"/>
-    <col min="10" max="10" width="11.8636363636364" customWidth="1"/>
-    <col min="11" max="11" width="20.6" customWidth="1"/>
-    <col min="12" max="12" width="8.6" customWidth="1"/>
-    <col min="13" max="13" width="4.6" customWidth="1"/>
-    <col min="14" max="14" width="5.26363636363636" customWidth="1"/>
-    <col min="15" max="15" width="10.2636363636364" customWidth="1"/>
-    <col min="16" max="16" width="7.86363636363636" customWidth="1"/>
+    <col min="6" max="6" width="6.3984375" customWidth="1"/>
+    <col min="7" max="7" width="8.265625" customWidth="1"/>
+    <col min="9" max="9" width="11.265625" customWidth="1"/>
+    <col min="10" max="10" width="11.86328125" customWidth="1"/>
+    <col min="11" max="11" width="20.59765625" customWidth="1"/>
+    <col min="12" max="12" width="8.59765625" customWidth="1"/>
+    <col min="13" max="13" width="4.59765625" customWidth="1"/>
+    <col min="14" max="14" width="5.265625" customWidth="1"/>
+    <col min="15" max="15" width="10.265625" customWidth="1"/>
+    <col min="16" max="16" width="7.86328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:16">
@@ -3564,63 +3044,61 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Y39"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="2" width="11.1363636363636" customWidth="1"/>
+    <col min="1" max="2" width="11.1328125" customWidth="1"/>
     <col min="3" max="5" width="14" customWidth="1"/>
-    <col min="6" max="8" width="11.8636363636364" customWidth="1"/>
-    <col min="9" max="9" width="20.2636363636364" customWidth="1"/>
-    <col min="10" max="10" width="15.6" customWidth="1"/>
-    <col min="11" max="11" width="20.2636363636364" customWidth="1"/>
-    <col min="12" max="12" width="15.6" customWidth="1"/>
-    <col min="13" max="13" width="20.2636363636364" customWidth="1"/>
-    <col min="14" max="14" width="15.6" customWidth="1"/>
-    <col min="15" max="15" width="18.8636363636364" customWidth="1"/>
-    <col min="16" max="16" width="4.4" customWidth="1"/>
-    <col min="17" max="17" width="8.13636363636364" customWidth="1"/>
-    <col min="20" max="20" width="18.1363636363636" customWidth="1"/>
+    <col min="6" max="8" width="11.86328125" customWidth="1"/>
+    <col min="9" max="9" width="20.265625" customWidth="1"/>
+    <col min="10" max="10" width="15.59765625" customWidth="1"/>
+    <col min="11" max="11" width="20.265625" customWidth="1"/>
+    <col min="12" max="12" width="15.59765625" customWidth="1"/>
+    <col min="13" max="13" width="20.265625" customWidth="1"/>
+    <col min="14" max="14" width="15.59765625" customWidth="1"/>
+    <col min="15" max="15" width="18.86328125" customWidth="1"/>
+    <col min="16" max="16" width="4.3984375" customWidth="1"/>
+    <col min="17" max="17" width="8.1328125" customWidth="1"/>
+    <col min="20" max="20" width="18.1328125" customWidth="1"/>
     <col min="21" max="21" width="24" customWidth="1"/>
-    <col min="22" max="22" width="4.6" customWidth="1"/>
-    <col min="23" max="23" width="4.13636363636364" customWidth="1"/>
-    <col min="24" max="24" width="7.72727272727273" customWidth="1"/>
-    <col min="25" max="25" width="7.13636363636364" customWidth="1"/>
+    <col min="22" max="22" width="4.59765625" customWidth="1"/>
+    <col min="23" max="23" width="4.1328125" customWidth="1"/>
+    <col min="24" max="24" width="7.73046875" customWidth="1"/>
+    <col min="25" max="25" width="7.1328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" spans="1:20">
+    <row r="1" spans="1:20" ht="33.75" customHeight="1">
       <c r="A1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="180" t="s">
         <v>30</v>
       </c>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="60" t="s">
+      <c r="D1" s="180"/>
+      <c r="E1" s="180"/>
+      <c r="F1" s="181" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="59"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="59" t="s">
+      <c r="G1" s="180"/>
+      <c r="H1" s="182"/>
+      <c r="I1" s="180" t="s">
         <v>32</v>
       </c>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="62" t="s">
+      <c r="J1" s="180"/>
+      <c r="K1" s="180"/>
+      <c r="L1" s="180"/>
+      <c r="M1" s="180"/>
+      <c r="N1" s="180"/>
+      <c r="O1" s="183" t="s">
         <v>33</v>
       </c>
-      <c r="P1" s="63"/>
-      <c r="Q1" s="63"/>
+      <c r="P1" s="59"/>
+      <c r="Q1" s="59"/>
       <c r="S1" t="s">
         <v>34</v>
       </c>
@@ -3629,953 +3107,953 @@
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="C2" s="64" t="s">
+      <c r="C2" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="64" t="s">
+      <c r="D2" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="E2" s="64" t="s">
+      <c r="E2" s="60" t="s">
         <v>36</v>
       </c>
-      <c r="F2" s="64" t="s">
+      <c r="F2" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="64" t="s">
+      <c r="G2" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="64" t="s">
+      <c r="H2" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="64" t="s">
+      <c r="I2" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="64" t="s">
+      <c r="J2" s="60" t="s">
         <v>39</v>
       </c>
-      <c r="K2" s="64" t="str">
+      <c r="K2" s="60" t="str">
         <f>I2</f>
         <v>input~GASNGA</v>
       </c>
-      <c r="L2" s="64" t="str">
+      <c r="L2" s="60" t="str">
         <f>J2</f>
         <v>input~ELC_gc</v>
       </c>
-      <c r="M2" s="64" t="str">
+      <c r="M2" s="60" t="str">
         <f>K2</f>
         <v>input~GASNGA</v>
       </c>
-      <c r="N2" s="64" t="str">
+      <c r="N2" s="60" t="str">
         <f>L2</f>
         <v>input~ELC_gc</v>
       </c>
-      <c r="O2" s="63"/>
-      <c r="P2" s="63"/>
-      <c r="Q2" s="63"/>
+      <c r="O2" s="184"/>
+      <c r="P2" s="59"/>
+      <c r="Q2" s="59"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="C3" s="64">
+      <c r="C3" s="60">
         <v>2020</v>
       </c>
-      <c r="D3" s="64">
+      <c r="D3" s="60">
         <v>2030</v>
       </c>
-      <c r="E3" s="64">
+      <c r="E3" s="60">
         <v>2050</v>
       </c>
-      <c r="F3" s="64">
+      <c r="F3" s="60">
         <f>C3</f>
         <v>2020</v>
       </c>
-      <c r="G3" s="64">
+      <c r="G3" s="60">
         <f t="shared" ref="G3:H3" si="0">D3</f>
         <v>2030</v>
       </c>
-      <c r="H3" s="64">
+      <c r="H3" s="60">
         <f t="shared" si="0"/>
         <v>2050</v>
       </c>
-      <c r="I3" s="64">
+      <c r="I3" s="60">
         <v>2015</v>
       </c>
-      <c r="J3" s="64">
+      <c r="J3" s="60">
         <v>2015</v>
       </c>
-      <c r="K3" s="64">
+      <c r="K3" s="60">
         <v>2030</v>
       </c>
-      <c r="L3" s="64">
+      <c r="L3" s="60">
         <v>2030</v>
       </c>
-      <c r="M3" s="64">
+      <c r="M3" s="60">
         <v>2050</v>
       </c>
-      <c r="N3" s="64">
+      <c r="N3" s="60">
         <v>2050</v>
       </c>
-      <c r="O3" s="63"/>
-      <c r="P3" s="63"/>
-      <c r="Q3" s="63"/>
-    </row>
-    <row r="4" ht="26" spans="1:20">
-      <c r="C4" s="65">
+      <c r="O3" s="184"/>
+      <c r="P3" s="59"/>
+      <c r="Q3" s="59"/>
+    </row>
+    <row r="4" spans="1:20" ht="26.25">
+      <c r="C4" s="61">
         <v>2020</v>
       </c>
-      <c r="D4" s="65">
+      <c r="D4" s="61">
         <v>2030</v>
       </c>
-      <c r="E4" s="65" t="s">
+      <c r="E4" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="66">
+      <c r="F4" s="62">
         <v>2015</v>
       </c>
-      <c r="G4" s="65">
+      <c r="G4" s="61">
         <v>2030</v>
       </c>
-      <c r="H4" s="67" t="s">
+      <c r="H4" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="I4" s="65" t="s">
+      <c r="I4" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="65" t="s">
+      <c r="J4" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="K4" s="68" t="s">
+      <c r="K4" s="64" t="s">
         <v>43</v>
       </c>
-      <c r="L4" s="69" t="s">
+      <c r="L4" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="65" t="s">
+      <c r="M4" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="N4" s="65" t="s">
+      <c r="N4" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="O4" s="70"/>
-      <c r="P4" s="63"/>
-      <c r="Q4" s="63"/>
+      <c r="O4" s="185"/>
+      <c r="P4" s="59"/>
+      <c r="Q4" s="59"/>
     </row>
     <row r="5" spans="1:20">
-      <c r="C5" s="71">
+      <c r="C5" s="66">
         <v>550</v>
       </c>
-      <c r="D5" s="71">
+      <c r="D5" s="66">
         <v>500</v>
       </c>
-      <c r="E5" s="71">
+      <c r="E5" s="66">
         <v>450</v>
       </c>
-      <c r="F5" s="72">
+      <c r="F5" s="67">
         <v>22</v>
       </c>
-      <c r="G5" s="73">
+      <c r="G5" s="68">
         <v>20</v>
       </c>
-      <c r="H5" s="74">
+      <c r="H5" s="69">
         <v>18</v>
       </c>
-      <c r="I5" s="75">
+      <c r="I5" s="70">
         <v>1.33</v>
       </c>
-      <c r="J5" s="75">
-        <v>0.094</v>
-      </c>
-      <c r="K5" s="76">
+      <c r="J5" s="70">
+        <v>9.4E-2</v>
+      </c>
+      <c r="K5" s="71">
         <v>1.3</v>
       </c>
-      <c r="L5" s="77">
-        <v>0.094</v>
-      </c>
-      <c r="M5" s="75">
+      <c r="L5" s="72">
+        <v>9.4E-2</v>
+      </c>
+      <c r="M5" s="70">
         <v>1.28</v>
       </c>
-      <c r="N5" s="75">
-        <v>0.094</v>
-      </c>
-      <c r="O5" s="78" t="s">
+      <c r="N5" s="70">
+        <v>9.4E-2</v>
+      </c>
+      <c r="O5" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="P5" s="79"/>
-      <c r="Q5" s="79"/>
+      <c r="P5" s="74"/>
+      <c r="Q5" s="74"/>
     </row>
     <row r="6" spans="1:20">
-      <c r="C6" s="80">
+      <c r="C6" s="75">
         <v>900</v>
       </c>
-      <c r="D6" s="80">
+      <c r="D6" s="75">
         <v>850</v>
       </c>
-      <c r="E6" s="80">
+      <c r="E6" s="75">
         <v>800</v>
       </c>
-      <c r="F6" s="81">
+      <c r="F6" s="76">
         <v>36</v>
       </c>
-      <c r="G6" s="82">
+      <c r="G6" s="77">
         <v>34</v>
       </c>
-      <c r="H6" s="83">
+      <c r="H6" s="78">
         <v>32</v>
       </c>
-      <c r="I6" s="84">
+      <c r="I6" s="79">
         <v>1.33</v>
       </c>
-      <c r="J6" s="84">
-        <v>1.094</v>
-      </c>
-      <c r="K6" s="85">
+      <c r="J6" s="79">
+        <v>1.0940000000000001</v>
+      </c>
+      <c r="K6" s="80">
         <v>1.3</v>
       </c>
-      <c r="L6" s="86">
-        <v>1.094</v>
-      </c>
-      <c r="M6" s="84">
+      <c r="L6" s="81">
+        <v>1.0940000000000001</v>
+      </c>
+      <c r="M6" s="79">
         <v>1.28</v>
       </c>
-      <c r="N6" s="84">
-        <v>1.094</v>
-      </c>
-      <c r="O6" s="87" t="s">
+      <c r="N6" s="79">
+        <v>1.0940000000000001</v>
+      </c>
+      <c r="O6" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="P6" s="88"/>
-      <c r="Q6" s="88"/>
+      <c r="P6" s="83"/>
+      <c r="Q6" s="83"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="C7" s="71">
+      <c r="C7" s="66">
         <v>1978</v>
       </c>
-      <c r="D7" s="71">
+      <c r="D7" s="66">
         <v>1598</v>
       </c>
-      <c r="E7" s="71">
+      <c r="E7" s="66">
         <v>1450</v>
       </c>
-      <c r="F7" s="72">
+      <c r="F7" s="67">
         <v>57</v>
       </c>
-      <c r="G7" s="73">
+      <c r="G7" s="68">
         <v>31</v>
       </c>
-      <c r="H7" s="74">
+      <c r="H7" s="69">
         <v>28</v>
       </c>
-      <c r="I7" s="75">
+      <c r="I7" s="70">
         <v>1.53</v>
       </c>
-      <c r="J7" s="75">
-        <v>0.094</v>
-      </c>
-      <c r="K7" s="76">
+      <c r="J7" s="70">
+        <v>9.4E-2</v>
+      </c>
+      <c r="K7" s="71">
         <v>1.47</v>
       </c>
-      <c r="L7" s="77">
-        <v>0.094</v>
-      </c>
-      <c r="M7" s="75">
+      <c r="L7" s="72">
+        <v>9.4E-2</v>
+      </c>
+      <c r="M7" s="70">
         <v>1.43</v>
       </c>
-      <c r="N7" s="75">
-        <v>0.094</v>
-      </c>
-      <c r="O7" s="78" t="s">
+      <c r="N7" s="70">
+        <v>9.4E-2</v>
+      </c>
+      <c r="O7" s="73" t="s">
         <v>49</v>
       </c>
-      <c r="P7" s="79"/>
-      <c r="Q7" s="79"/>
+      <c r="P7" s="74"/>
+      <c r="Q7" s="74"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="C8" s="89">
+      <c r="C8" s="84">
         <v>1610</v>
       </c>
-      <c r="D8" s="89">
+      <c r="D8" s="84">
         <v>740</v>
       </c>
-      <c r="E8" s="89">
+      <c r="E8" s="84">
         <v>200</v>
       </c>
-      <c r="F8" s="81">
+      <c r="F8" s="76">
         <v>49</v>
       </c>
-      <c r="G8" s="82">
+      <c r="G8" s="77">
         <v>15</v>
       </c>
-      <c r="H8" s="83">
+      <c r="H8" s="78">
         <v>10</v>
       </c>
-      <c r="I8" s="84">
+      <c r="I8" s="79">
         <v>0</v>
       </c>
-      <c r="J8" s="84">
+      <c r="J8" s="79">
         <v>1.39</v>
       </c>
-      <c r="K8" s="85">
+      <c r="K8" s="80">
         <v>0</v>
       </c>
-      <c r="L8" s="86">
+      <c r="L8" s="81">
         <v>1.19</v>
       </c>
-      <c r="M8" s="84">
+      <c r="M8" s="79">
         <v>0</v>
       </c>
-      <c r="N8" s="84">
+      <c r="N8" s="79">
         <v>1.17</v>
       </c>
-      <c r="O8" s="87" t="s">
+      <c r="O8" s="82" t="s">
         <v>50</v>
       </c>
-      <c r="P8" s="88"/>
-      <c r="Q8" s="88"/>
+      <c r="P8" s="83"/>
+      <c r="Q8" s="83"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="C9" s="90">
+      <c r="C9" s="85">
         <v>2530</v>
       </c>
-      <c r="D9" s="90">
+      <c r="D9" s="85">
         <v>1175</v>
       </c>
-      <c r="E9" s="90">
+      <c r="E9" s="85">
         <v>350</v>
       </c>
-      <c r="F9" s="72">
+      <c r="F9" s="67">
         <v>77</v>
       </c>
-      <c r="G9" s="73">
+      <c r="G9" s="68">
         <v>34</v>
       </c>
-      <c r="H9" s="74">
+      <c r="H9" s="69">
         <v>18</v>
       </c>
-      <c r="I9" s="75">
+      <c r="I9" s="70">
         <v>0</v>
       </c>
-      <c r="J9" s="75">
+      <c r="J9" s="70">
         <v>1.5</v>
       </c>
-      <c r="K9" s="76">
+      <c r="K9" s="71">
         <v>0</v>
       </c>
-      <c r="L9" s="77">
+      <c r="L9" s="72">
         <v>1.25</v>
       </c>
-      <c r="M9" s="75">
+      <c r="M9" s="70">
         <v>0</v>
       </c>
-      <c r="N9" s="75">
+      <c r="N9" s="70">
         <v>1.19</v>
       </c>
-      <c r="O9" s="78" t="s">
+      <c r="O9" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="P9" s="79"/>
-      <c r="Q9" s="79"/>
+      <c r="P9" s="74"/>
+      <c r="Q9" s="74"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="C10" s="89">
+      <c r="C10" s="84">
         <v>1265</v>
       </c>
-      <c r="D10" s="89">
+      <c r="D10" s="84">
         <v>600</v>
       </c>
-      <c r="E10" s="89">
+      <c r="E10" s="84">
         <v>180</v>
       </c>
-      <c r="F10" s="81">
+      <c r="F10" s="76">
         <v>28</v>
       </c>
-      <c r="G10" s="82">
+      <c r="G10" s="77">
         <v>14</v>
       </c>
-      <c r="H10" s="83">
+      <c r="H10" s="78">
         <v>9</v>
       </c>
-      <c r="I10" s="84">
+      <c r="I10" s="79">
         <v>0</v>
       </c>
-      <c r="J10" s="84">
+      <c r="J10" s="79">
         <v>1.3952</v>
       </c>
-      <c r="K10" s="85">
+      <c r="K10" s="80">
         <v>0</v>
       </c>
-      <c r="L10" s="86">
+      <c r="L10" s="81">
         <v>1.268</v>
       </c>
-      <c r="M10" s="84">
+      <c r="M10" s="79">
         <v>0</v>
       </c>
-      <c r="N10" s="84">
+      <c r="N10" s="79">
         <v>1.18</v>
       </c>
-      <c r="O10" s="87" t="s">
+      <c r="O10" s="82" t="s">
         <v>52</v>
       </c>
-      <c r="P10" s="88"/>
-      <c r="Q10" s="88"/>
+      <c r="P10" s="83"/>
+      <c r="Q10" s="83"/>
     </row>
     <row r="11" spans="1:20">
-      <c r="C11" s="90">
+      <c r="C11" s="85">
         <v>1897.5</v>
       </c>
-      <c r="D11" s="90">
+      <c r="D11" s="85">
         <v>715</v>
       </c>
-      <c r="E11" s="90">
+      <c r="E11" s="85">
         <v>300</v>
       </c>
-      <c r="F11" s="72">
+      <c r="F11" s="67">
         <v>41</v>
       </c>
-      <c r="G11" s="73">
+      <c r="G11" s="68">
         <v>17</v>
       </c>
-      <c r="H11" s="74">
+      <c r="H11" s="69">
         <v>15</v>
       </c>
-      <c r="I11" s="75">
+      <c r="I11" s="70">
         <v>0</v>
       </c>
-      <c r="J11" s="75">
+      <c r="J11" s="70">
         <v>1.3952</v>
       </c>
-      <c r="K11" s="76">
+      <c r="K11" s="71">
         <v>0</v>
       </c>
-      <c r="L11" s="77">
+      <c r="L11" s="72">
         <v>1.268</v>
       </c>
-      <c r="M11" s="75">
+      <c r="M11" s="70">
         <v>0</v>
       </c>
-      <c r="N11" s="75">
+      <c r="N11" s="70">
         <v>1.2</v>
       </c>
-      <c r="O11" s="78" t="s">
+      <c r="O11" s="73" t="s">
         <v>53</v>
       </c>
-      <c r="P11" s="79"/>
-      <c r="Q11" s="79"/>
+      <c r="P11" s="74"/>
+      <c r="Q11" s="74"/>
     </row>
     <row r="12" spans="1:20">
-      <c r="C12" s="89">
-        <v>3332.08823529412</v>
-      </c>
-      <c r="D12" s="89">
+      <c r="C12" s="84">
+        <v>3332.0882352941198</v>
+      </c>
+      <c r="D12" s="84">
         <v>1421.39215686275</v>
       </c>
-      <c r="E12" s="89">
+      <c r="E12" s="84">
         <v>600</v>
       </c>
-      <c r="F12" s="81">
-        <v>55.825</v>
-      </c>
-      <c r="G12" s="82">
+      <c r="F12" s="76">
+        <v>55.825000000000003</v>
+      </c>
+      <c r="G12" s="77">
         <v>36.18</v>
       </c>
-      <c r="H12" s="83">
+      <c r="H12" s="78">
         <v>39</v>
       </c>
-      <c r="I12" s="84">
-        <v>1.99666703875969</v>
-      </c>
-      <c r="J12" s="84">
-        <v>0.83712</v>
-      </c>
-      <c r="K12" s="85">
+      <c r="I12" s="79">
+        <v>1.9966670387596901</v>
+      </c>
+      <c r="J12" s="79">
+        <v>0.83711999999999998</v>
+      </c>
+      <c r="K12" s="80">
         <v>1.45562727909392</v>
       </c>
-      <c r="L12" s="86">
-        <v>0.7608</v>
-      </c>
-      <c r="M12" s="84">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="N12" s="84">
-        <v>0.708</v>
-      </c>
-      <c r="O12" s="87" t="s">
+      <c r="L12" s="81">
+        <v>0.76080000000000003</v>
+      </c>
+      <c r="M12" s="79">
+        <v>0.33333333333333298</v>
+      </c>
+      <c r="N12" s="79">
+        <v>0.70799999999999996</v>
+      </c>
+      <c r="O12" s="82" t="s">
         <v>54</v>
       </c>
-      <c r="P12" s="88"/>
-      <c r="Q12" s="88"/>
+      <c r="P12" s="83"/>
+      <c r="Q12" s="83"/>
     </row>
     <row r="13" spans="1:20">
-      <c r="C13" s="90">
-        <v>5331.34117647059</v>
-      </c>
-      <c r="D13" s="90">
-        <v>2920.89411764706</v>
-      </c>
-      <c r="E13" s="90">
+      <c r="C13" s="85">
+        <v>5331.3411764705897</v>
+      </c>
+      <c r="D13" s="85">
+        <v>2920.8941176470598</v>
+      </c>
+      <c r="E13" s="85">
         <v>1100</v>
       </c>
-      <c r="F13" s="72">
-        <v>94.9025</v>
-      </c>
-      <c r="G13" s="73">
-        <v>63.315</v>
-      </c>
-      <c r="H13" s="74">
+      <c r="F13" s="67">
+        <v>94.902500000000003</v>
+      </c>
+      <c r="G13" s="68">
+        <v>63.314999999999998</v>
+      </c>
+      <c r="H13" s="69">
         <v>48.75</v>
       </c>
-      <c r="I13" s="75">
-        <v>1.99666703875969</v>
-      </c>
-      <c r="J13" s="75">
-        <v>0.83712</v>
-      </c>
-      <c r="K13" s="76">
+      <c r="I13" s="70">
+        <v>1.9966670387596901</v>
+      </c>
+      <c r="J13" s="70">
+        <v>0.83711999999999998</v>
+      </c>
+      <c r="K13" s="71">
         <v>1.45562727909392</v>
       </c>
-      <c r="L13" s="77">
-        <v>0.7608</v>
-      </c>
-      <c r="M13" s="75">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="N13" s="75">
+      <c r="L13" s="72">
+        <v>0.76080000000000003</v>
+      </c>
+      <c r="M13" s="70">
+        <v>0.33333333333333298</v>
+      </c>
+      <c r="N13" s="70">
         <v>0.72</v>
       </c>
-      <c r="O13" s="78" t="s">
+      <c r="O13" s="73" t="s">
         <v>55</v>
       </c>
-      <c r="P13" s="79"/>
-      <c r="Q13" s="79"/>
+      <c r="P13" s="74"/>
+      <c r="Q13" s="74"/>
     </row>
     <row r="14" spans="1:20">
-      <c r="C14" s="91">
+      <c r="C14" s="86">
         <v>1200</v>
       </c>
-      <c r="D14" s="91">
+      <c r="D14" s="86">
         <v>733</v>
       </c>
-      <c r="E14" s="91">
+      <c r="E14" s="86">
         <v>263</v>
       </c>
-      <c r="F14" s="92">
+      <c r="F14" s="87">
         <v>42</v>
       </c>
-      <c r="G14" s="93">
+      <c r="G14" s="88">
         <v>22</v>
       </c>
-      <c r="H14" s="94">
+      <c r="H14" s="89">
         <v>9</v>
       </c>
-      <c r="I14" s="95">
+      <c r="I14" s="90">
         <v>0</v>
       </c>
-      <c r="J14" s="96">
+      <c r="J14" s="91">
         <v>0.01</v>
       </c>
-      <c r="K14" s="97">
+      <c r="K14" s="92">
         <v>0</v>
       </c>
-      <c r="L14" s="98">
+      <c r="L14" s="93">
         <v>0.01</v>
       </c>
-      <c r="M14" s="96">
+      <c r="M14" s="91">
         <v>0</v>
       </c>
-      <c r="N14" s="96">
+      <c r="N14" s="91">
         <v>0.01</v>
       </c>
-      <c r="O14" s="99" t="s">
+      <c r="O14" s="94" t="s">
         <v>56</v>
       </c>
-      <c r="P14" s="100"/>
-      <c r="Q14" s="100"/>
+      <c r="P14" s="95"/>
+      <c r="Q14" s="95"/>
     </row>
     <row r="15" spans="1:20">
-      <c r="C15" s="101">
+      <c r="C15" s="96">
         <v>450</v>
       </c>
-      <c r="D15" s="101">
+      <c r="D15" s="96">
         <v>450</v>
       </c>
-      <c r="E15" s="101">
+      <c r="E15" s="96">
         <v>450</v>
       </c>
-      <c r="F15" s="102">
+      <c r="F15" s="97">
         <v>18</v>
       </c>
-      <c r="G15" s="103">
+      <c r="G15" s="98">
         <v>18</v>
       </c>
-      <c r="H15" s="104">
+      <c r="H15" s="99">
         <v>18</v>
       </c>
-      <c r="I15" s="105">
+      <c r="I15" s="100">
         <v>0.265822784810126</v>
       </c>
-      <c r="J15" s="106">
+      <c r="J15" s="101">
         <v>0.06</v>
       </c>
-      <c r="K15" s="107">
+      <c r="K15" s="102">
         <v>0.265822784810126</v>
       </c>
-      <c r="L15" s="108">
+      <c r="L15" s="103">
         <v>0.06</v>
       </c>
-      <c r="M15" s="106">
+      <c r="M15" s="101">
         <v>0.265822784810126</v>
       </c>
-      <c r="N15" s="106">
+      <c r="N15" s="101">
         <v>0.06</v>
       </c>
-      <c r="O15" s="109" t="s">
+      <c r="O15" s="104" t="s">
         <v>57</v>
       </c>
-      <c r="P15" s="110"/>
-      <c r="Q15" s="110"/>
+      <c r="P15" s="105"/>
+      <c r="Q15" s="105"/>
     </row>
     <row r="16" spans="1:20">
-      <c r="C16" s="111">
+      <c r="C16" s="106">
         <v>200</v>
       </c>
-      <c r="D16" s="111">
+      <c r="D16" s="106">
         <v>200</v>
       </c>
-      <c r="E16" s="111">
+      <c r="E16" s="106">
         <v>200</v>
       </c>
-      <c r="F16" s="112">
+      <c r="F16" s="107">
         <v>20</v>
       </c>
-      <c r="G16" s="113">
+      <c r="G16" s="108">
         <v>20</v>
       </c>
-      <c r="H16" s="114">
+      <c r="H16" s="109">
         <v>20</v>
       </c>
-      <c r="I16" s="115">
-        <v>0.013</v>
-      </c>
-      <c r="J16" s="116">
-        <v>0.036</v>
-      </c>
-      <c r="K16" s="117">
-        <v>0.013</v>
-      </c>
-      <c r="L16" s="118">
-        <v>0.036</v>
-      </c>
-      <c r="M16" s="116">
-        <v>0.013</v>
-      </c>
-      <c r="N16" s="116">
-        <v>0.036</v>
-      </c>
-      <c r="O16" s="119" t="s">
+      <c r="I16" s="110">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="J16" s="111">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="K16" s="112">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="L16" s="113">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="M16" s="111">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="N16" s="111">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="O16" s="114" t="s">
         <v>58</v>
       </c>
-      <c r="P16" s="120"/>
-      <c r="Q16" s="120"/>
+      <c r="P16" s="115"/>
+      <c r="Q16" s="115"/>
     </row>
     <row r="17" spans="1:25">
-      <c r="C17" s="101">
+      <c r="C17" s="96">
         <v>175</v>
       </c>
-      <c r="D17" s="101">
+      <c r="D17" s="96">
         <v>175</v>
       </c>
-      <c r="E17" s="101">
+      <c r="E17" s="96">
         <v>175</v>
       </c>
-      <c r="F17" s="102">
+      <c r="F17" s="97">
         <v>5</v>
       </c>
-      <c r="G17" s="103">
+      <c r="G17" s="98">
         <v>5</v>
       </c>
-      <c r="H17" s="104">
+      <c r="H17" s="99">
         <v>5</v>
       </c>
-      <c r="I17" s="105">
-        <v>0.014</v>
-      </c>
-      <c r="J17" s="106">
+      <c r="I17" s="100">
+        <v>1.4E-2</v>
+      </c>
+      <c r="J17" s="101">
         <v>0</v>
       </c>
-      <c r="K17" s="107">
-        <v>0.014</v>
-      </c>
-      <c r="L17" s="108">
+      <c r="K17" s="102">
+        <v>1.4E-2</v>
+      </c>
+      <c r="L17" s="103">
         <v>0</v>
       </c>
-      <c r="M17" s="106">
-        <v>0.014</v>
-      </c>
-      <c r="N17" s="106">
+      <c r="M17" s="101">
+        <v>1.4E-2</v>
+      </c>
+      <c r="N17" s="101">
         <v>0</v>
       </c>
-      <c r="O17" s="109" t="s">
+      <c r="O17" s="104" t="s">
         <v>59</v>
       </c>
-      <c r="P17" s="110"/>
-      <c r="Q17" s="110"/>
+      <c r="P17" s="105"/>
+      <c r="Q17" s="105"/>
     </row>
     <row r="18" spans="1:25">
-      <c r="C18" s="121">
+      <c r="C18" s="116">
         <v>1000</v>
       </c>
-      <c r="D18" s="121">
+      <c r="D18" s="116">
         <v>720</v>
       </c>
-      <c r="E18" s="121">
+      <c r="E18" s="116">
         <v>364</v>
       </c>
-      <c r="F18" s="122">
+      <c r="F18" s="117">
         <v>50</v>
       </c>
-      <c r="G18" s="123">
+      <c r="G18" s="118">
         <v>31</v>
       </c>
-      <c r="H18" s="124">
+      <c r="H18" s="119">
         <v>18</v>
       </c>
-      <c r="I18" s="125">
+      <c r="I18" s="120">
         <v>0.2389</v>
       </c>
-      <c r="J18" s="126">
-        <v>0.03056</v>
-      </c>
-      <c r="K18" s="127">
+      <c r="J18" s="121">
+        <v>3.056E-2</v>
+      </c>
+      <c r="K18" s="122">
         <v>0.2389</v>
       </c>
-      <c r="L18" s="128">
-        <v>0.03056</v>
-      </c>
-      <c r="M18" s="126">
+      <c r="L18" s="123">
+        <v>3.056E-2</v>
+      </c>
+      <c r="M18" s="121">
         <v>0.2389</v>
       </c>
-      <c r="N18" s="126">
-        <v>0.03056</v>
-      </c>
-      <c r="O18" s="129" t="s">
+      <c r="N18" s="121">
+        <v>3.056E-2</v>
+      </c>
+      <c r="O18" s="124" t="s">
         <v>60</v>
       </c>
-      <c r="P18" s="130"/>
-      <c r="Q18" s="130"/>
+      <c r="P18" s="125"/>
+      <c r="Q18" s="125"/>
     </row>
     <row r="19" spans="1:25">
-      <c r="C19" s="131">
+      <c r="C19" s="126">
         <v>1556</v>
       </c>
-      <c r="D19" s="131">
+      <c r="D19" s="126">
         <v>1143</v>
       </c>
-      <c r="E19" s="132">
+      <c r="E19" s="127">
         <v>673</v>
       </c>
-      <c r="F19" s="133">
+      <c r="F19" s="128">
         <v>54</v>
       </c>
-      <c r="G19" s="134">
+      <c r="G19" s="129">
         <v>40</v>
       </c>
-      <c r="H19" s="135">
+      <c r="H19" s="130">
         <v>24</v>
       </c>
-      <c r="I19" s="136">
-        <v>0.035</v>
-      </c>
-      <c r="J19" s="137">
+      <c r="I19" s="131">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="J19" s="132">
         <v>0.02</v>
       </c>
-      <c r="K19" s="138">
-        <v>0.035</v>
-      </c>
-      <c r="L19" s="139">
+      <c r="K19" s="133">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="L19" s="134">
         <v>0.02</v>
       </c>
-      <c r="M19" s="137">
-        <v>0.035</v>
-      </c>
-      <c r="N19" s="137">
+      <c r="M19" s="132">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="N19" s="132">
         <v>0.02</v>
       </c>
-      <c r="O19" s="140" t="s">
+      <c r="O19" s="135" t="s">
         <v>61</v>
       </c>
-      <c r="P19" s="141"/>
-      <c r="Q19" s="141"/>
+      <c r="P19" s="136"/>
+      <c r="Q19" s="136"/>
     </row>
     <row r="20" spans="1:25">
-      <c r="C20" s="142">
+      <c r="C20" s="137">
         <v>2332</v>
       </c>
-      <c r="D20" s="142">
+      <c r="D20" s="137">
         <v>1511</v>
       </c>
-      <c r="E20" s="142">
+      <c r="E20" s="137">
         <v>965</v>
       </c>
-      <c r="F20" s="143">
+      <c r="F20" s="138">
         <v>163</v>
       </c>
-      <c r="G20" s="144">
+      <c r="G20" s="139">
         <v>106</v>
       </c>
-      <c r="H20" s="145">
+      <c r="H20" s="140">
         <v>68</v>
       </c>
-      <c r="I20" s="146">
-        <v>0.463266666666667</v>
-      </c>
-      <c r="J20" s="147">
+      <c r="I20" s="141">
+        <v>0.46326666666666699</v>
+      </c>
+      <c r="J20" s="142">
         <v>1.91881040892193</v>
       </c>
-      <c r="K20" s="148">
-        <v>0.39244195142278</v>
-      </c>
-      <c r="L20" s="149">
+      <c r="K20" s="143">
+        <v>0.39244195142277999</v>
+      </c>
+      <c r="L20" s="144">
         <v>1.60098120886331</v>
       </c>
-      <c r="M20" s="147">
+      <c r="M20" s="142">
         <v>0.37890902062421</v>
       </c>
-      <c r="N20" s="147">
-        <v>1.56940834539103</v>
-      </c>
-      <c r="O20" s="150" t="s">
+      <c r="N20" s="142">
+        <v>1.5694083453910299</v>
+      </c>
+      <c r="O20" s="145" t="s">
         <v>62</v>
       </c>
-      <c r="P20" s="130"/>
-      <c r="Q20" s="130"/>
+      <c r="P20" s="125"/>
+      <c r="Q20" s="125"/>
     </row>
     <row r="21" spans="1:25">
-      <c r="C21" s="151">
-        <v>769.876819708847</v>
-      </c>
-      <c r="D21" s="151">
-        <v>648.044461034383</v>
-      </c>
-      <c r="E21" s="151">
-        <v>518.290592438013</v>
-      </c>
-      <c r="F21" s="152">
+      <c r="C21" s="146">
+        <v>769.87681970884705</v>
+      </c>
+      <c r="D21" s="146">
+        <v>648.04446103438295</v>
+      </c>
+      <c r="E21" s="146">
+        <v>518.29059243801305</v>
+      </c>
+      <c r="F21" s="147">
         <v>26.9456886898096</v>
       </c>
-      <c r="G21" s="153">
-        <v>22.6815561362034</v>
-      </c>
-      <c r="H21" s="154">
+      <c r="G21" s="148">
+        <v>22.681556136203401</v>
+      </c>
+      <c r="H21" s="149">
         <v>18.1401707353305</v>
       </c>
-      <c r="I21" s="155">
-        <v>2.77777777777778</v>
-      </c>
-      <c r="J21" s="156">
-        <v>2.22222222222222</v>
-      </c>
-      <c r="K21" s="157">
-        <v>1.66666666666667</v>
-      </c>
-      <c r="L21" s="158">
-        <v>1.38888888888889</v>
-      </c>
-      <c r="M21" s="156">
-        <v>1.13888888888889</v>
-      </c>
-      <c r="N21" s="156">
+      <c r="I21" s="150">
+        <v>2.7777777777777799</v>
+      </c>
+      <c r="J21" s="151">
+        <v>2.2222222222222201</v>
+      </c>
+      <c r="K21" s="152">
+        <v>1.6666666666666701</v>
+      </c>
+      <c r="L21" s="153">
+        <v>1.3888888888888899</v>
+      </c>
+      <c r="M21" s="151">
+        <v>1.1388888888888899</v>
+      </c>
+      <c r="N21" s="151">
         <v>0.3</v>
       </c>
-      <c r="O21" s="159" t="s">
+      <c r="O21" s="154" t="s">
         <v>63</v>
       </c>
-      <c r="P21" s="160"/>
-      <c r="Q21" s="160"/>
+      <c r="P21" s="155"/>
+      <c r="Q21" s="155"/>
     </row>
     <row r="22" spans="1:25">
-      <c r="C22" s="161">
-        <v>1259.79843225084</v>
-      </c>
-      <c r="D22" s="161">
-        <v>894.301356227448</v>
-      </c>
-      <c r="E22" s="161">
+      <c r="C22" s="156">
+        <v>1259.7984322508401</v>
+      </c>
+      <c r="D22" s="156">
+        <v>894.30135622744797</v>
+      </c>
+      <c r="E22" s="156">
         <v>495</v>
       </c>
-      <c r="F22" s="162">
-        <v>44.0929451287794</v>
-      </c>
-      <c r="G22" s="163">
-        <v>31.3005474679607</v>
-      </c>
-      <c r="H22" s="164">
-        <v>17.325</v>
-      </c>
-      <c r="I22" s="165">
+      <c r="F22" s="157">
+        <v>44.092945128779398</v>
+      </c>
+      <c r="G22" s="158">
+        <v>31.300547467960701</v>
+      </c>
+      <c r="H22" s="159">
+        <v>17.324999999999999</v>
+      </c>
+      <c r="I22" s="160">
         <v>2</v>
       </c>
-      <c r="J22" s="166">
+      <c r="J22" s="161">
         <v>0.3</v>
       </c>
-      <c r="K22" s="167">
+      <c r="K22" s="162">
         <v>1.80555555555556</v>
       </c>
-      <c r="L22" s="168">
+      <c r="L22" s="163">
         <v>0.3</v>
       </c>
-      <c r="M22" s="166">
+      <c r="M22" s="161">
         <v>1.5</v>
       </c>
-      <c r="N22" s="166">
+      <c r="N22" s="161">
         <v>0.3</v>
       </c>
-      <c r="O22" s="169" t="s">
+      <c r="O22" s="164" t="s">
         <v>64</v>
       </c>
-      <c r="P22" s="170"/>
-      <c r="Q22" s="170"/>
+      <c r="P22" s="165"/>
+      <c r="Q22" s="165"/>
     </row>
     <row r="23" spans="1:25">
-      <c r="C23" s="171">
+      <c r="C23" s="166">
         <v>174</v>
       </c>
-      <c r="D23" s="171">
+      <c r="D23" s="166">
         <v>174</v>
       </c>
-      <c r="E23" s="171">
+      <c r="E23" s="166">
         <v>174</v>
       </c>
-      <c r="F23" s="172">
+      <c r="F23" s="167">
         <v>3</v>
       </c>
-      <c r="G23" s="173">
+      <c r="G23" s="168">
         <v>3</v>
       </c>
-      <c r="H23" s="174">
+      <c r="H23" s="169">
         <v>3</v>
       </c>
-      <c r="I23" s="175">
+      <c r="I23" s="170">
         <v>0</v>
       </c>
-      <c r="J23" s="176">
-        <v>0.205882352941176</v>
-      </c>
-      <c r="K23" s="177">
+      <c r="J23" s="171">
+        <v>0.20588235294117599</v>
+      </c>
+      <c r="K23" s="172">
         <v>0</v>
       </c>
-      <c r="L23" s="178">
-        <v>0.205882352941176</v>
-      </c>
-      <c r="M23" s="176">
+      <c r="L23" s="173">
+        <v>0.20588235294117599</v>
+      </c>
+      <c r="M23" s="171">
         <v>0</v>
       </c>
-      <c r="N23" s="176">
-        <v>0.205882352941176</v>
-      </c>
-      <c r="O23" s="179" t="s">
+      <c r="N23" s="171">
+        <v>0.20588235294117599</v>
+      </c>
+      <c r="O23" s="174" t="s">
         <v>65</v>
       </c>
-      <c r="P23" s="160"/>
-      <c r="Q23" s="160"/>
-    </row>
-    <row r="26" ht="17.75" spans="1:25">
+      <c r="P23" s="155"/>
+      <c r="Q23" s="155"/>
+    </row>
+    <row r="26" spans="1:25" ht="16.899999999999999">
       <c r="C26" s="53" t="s">
         <v>66</v>
       </c>
@@ -4583,7 +4061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" ht="15.25" spans="1:25">
+    <row r="27" spans="1:25">
       <c r="A27" s="54" t="s">
         <v>4</v>
       </c>
@@ -4706,7 +4184,7 @@
       </c>
       <c r="J28" s="9">
         <f t="shared" si="2"/>
-        <v>0.094</v>
+        <v>9.4E-2</v>
       </c>
       <c r="K28" s="9">
         <f t="shared" si="2"/>
@@ -4714,7 +4192,7 @@
       </c>
       <c r="L28" s="9">
         <f t="shared" si="2"/>
-        <v>0.094</v>
+        <v>9.4E-2</v>
       </c>
       <c r="M28" s="9">
         <f t="shared" si="2"/>
@@ -4722,16 +4200,16 @@
       </c>
       <c r="N28" s="9">
         <f t="shared" si="2"/>
-        <v>0.094</v>
-      </c>
-      <c r="O28" s="180" t="s">
+        <v>9.4E-2</v>
+      </c>
+      <c r="O28" s="175" t="s">
         <v>70</v>
       </c>
       <c r="P28">
         <v>25</v>
       </c>
       <c r="Q28">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="S28" t="str">
         <f>IF(O28="","*","PRE")</f>
@@ -4793,25 +4271,25 @@
         <f t="shared" si="4"/>
         <v>1.33</v>
       </c>
-      <c r="J29" s="181">
+      <c r="J29" s="176">
         <f t="shared" si="4"/>
-        <v>1.094</v>
+        <v>1.0940000000000001</v>
       </c>
       <c r="K29" s="9">
         <f t="shared" si="4"/>
         <v>1.3</v>
       </c>
-      <c r="L29" s="181">
+      <c r="L29" s="176">
         <f t="shared" si="4"/>
-        <v>1.094</v>
+        <v>1.0940000000000001</v>
       </c>
       <c r="M29" s="9">
         <f t="shared" si="4"/>
         <v>1.28</v>
       </c>
-      <c r="N29" s="181">
+      <c r="N29" s="176">
         <f t="shared" si="4"/>
-        <v>1.094</v>
+        <v>1.0940000000000001</v>
       </c>
       <c r="O29" t="s">
         <v>73</v>
@@ -4820,7 +4298,7 @@
         <v>25</v>
       </c>
       <c r="Q29">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="S29" t="str">
         <f t="shared" ref="S29:S39" si="5">IF(O29="","*","PRE")</f>
@@ -4884,7 +4362,7 @@
       </c>
       <c r="J30" s="9">
         <f t="shared" si="7"/>
-        <v>0.094</v>
+        <v>9.4E-2</v>
       </c>
       <c r="K30" s="9">
         <f t="shared" si="7"/>
@@ -4892,7 +4370,7 @@
       </c>
       <c r="L30" s="9">
         <f t="shared" si="7"/>
-        <v>0.094</v>
+        <v>9.4E-2</v>
       </c>
       <c r="M30" s="9">
         <f t="shared" si="7"/>
@@ -4900,9 +4378,9 @@
       </c>
       <c r="N30" s="9">
         <f t="shared" si="7"/>
-        <v>0.094</v>
-      </c>
-      <c r="O30" s="180" t="s">
+        <v>9.4E-2</v>
+      </c>
+      <c r="O30" s="175" t="s">
         <v>70</v>
       </c>
       <c r="S30" t="str">
@@ -4983,7 +4461,7 @@
         <v>25</v>
       </c>
       <c r="Q31">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="S31" t="str">
         <f t="shared" si="5"/>
@@ -5056,7 +4534,7 @@
         <f t="shared" si="9"/>
         <v>1.19</v>
       </c>
-      <c r="O32" s="180" t="s">
+      <c r="O32" s="175" t="s">
         <v>70</v>
       </c>
       <c r="S32" t="str">
@@ -5137,7 +4615,7 @@
         <v>25</v>
       </c>
       <c r="Q33">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="S33" t="str">
         <f t="shared" si="5"/>
@@ -5210,7 +4688,7 @@
         <f t="shared" si="11"/>
         <v>1.2</v>
       </c>
-      <c r="O34" s="180" t="s">
+      <c r="O34" s="175" t="s">
         <v>70</v>
       </c>
       <c r="S34" t="str">
@@ -5247,7 +4725,7 @@
       </c>
       <c r="C35" s="38">
         <f t="shared" ref="C35:N35" si="12">C12</f>
-        <v>3332.08823529412</v>
+        <v>3332.0882352941198</v>
       </c>
       <c r="D35" s="38">
         <f t="shared" si="12"/>
@@ -5259,7 +4737,7 @@
       </c>
       <c r="F35" s="38">
         <f t="shared" si="12"/>
-        <v>55.825</v>
+        <v>55.825000000000003</v>
       </c>
       <c r="G35" s="38">
         <f t="shared" si="12"/>
@@ -5271,11 +4749,11 @@
       </c>
       <c r="I35" s="9">
         <f t="shared" si="12"/>
-        <v>1.99666703875969</v>
+        <v>1.9966670387596901</v>
       </c>
       <c r="J35" s="9">
         <f t="shared" si="12"/>
-        <v>0.83712</v>
+        <v>0.83711999999999998</v>
       </c>
       <c r="K35" s="9">
         <f t="shared" si="12"/>
@@ -5283,15 +4761,15 @@
       </c>
       <c r="L35" s="9">
         <f t="shared" si="12"/>
-        <v>0.7608</v>
+        <v>0.76080000000000003</v>
       </c>
       <c r="M35" s="9">
         <f t="shared" si="12"/>
-        <v>0.333333333333333</v>
+        <v>0.33333333333333298</v>
       </c>
       <c r="N35" s="9">
         <f t="shared" si="12"/>
-        <v>0.708</v>
+        <v>0.70799999999999996</v>
       </c>
       <c r="O35" t="s">
         <v>76</v>
@@ -5300,7 +4778,7 @@
         <v>25</v>
       </c>
       <c r="Q35">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="S35" t="str">
         <f t="shared" si="5"/>
@@ -5330,11 +4808,11 @@
     <row r="36" spans="1:25">
       <c r="C36" s="38">
         <f t="shared" ref="C36:N36" si="13">C13</f>
-        <v>5331.34117647059</v>
+        <v>5331.3411764705897</v>
       </c>
       <c r="D36" s="38">
         <f t="shared" si="13"/>
-        <v>2920.89411764706</v>
+        <v>2920.8941176470598</v>
       </c>
       <c r="E36" s="38">
         <f t="shared" si="13"/>
@@ -5342,11 +4820,11 @@
       </c>
       <c r="F36" s="38">
         <f t="shared" si="13"/>
-        <v>94.9025</v>
+        <v>94.902500000000003</v>
       </c>
       <c r="G36" s="38">
         <f t="shared" si="13"/>
-        <v>63.315</v>
+        <v>63.314999999999998</v>
       </c>
       <c r="H36" s="38">
         <f t="shared" si="13"/>
@@ -5354,11 +4832,11 @@
       </c>
       <c r="I36" s="9">
         <f t="shared" si="13"/>
-        <v>1.99666703875969</v>
+        <v>1.9966670387596901</v>
       </c>
       <c r="J36" s="9">
         <f t="shared" si="13"/>
-        <v>0.83712</v>
+        <v>0.83711999999999998</v>
       </c>
       <c r="K36" s="9">
         <f t="shared" si="13"/>
@@ -5366,17 +4844,17 @@
       </c>
       <c r="L36" s="9">
         <f t="shared" si="13"/>
-        <v>0.7608</v>
+        <v>0.76080000000000003</v>
       </c>
       <c r="M36" s="9">
         <f t="shared" si="13"/>
-        <v>0.333333333333333</v>
+        <v>0.33333333333333298</v>
       </c>
       <c r="N36" s="9">
         <f t="shared" si="13"/>
         <v>0.72</v>
       </c>
-      <c r="O36" s="180" t="s">
+      <c r="O36" s="175" t="s">
         <v>70</v>
       </c>
       <c r="S36" t="str">
@@ -5407,15 +4885,15 @@
     <row r="37" spans="1:25">
       <c r="C37" s="38">
         <f t="shared" ref="C37:N37" si="14">C21</f>
-        <v>769.876819708847</v>
+        <v>769.87681970884705</v>
       </c>
       <c r="D37" s="38">
         <f t="shared" si="14"/>
-        <v>648.044461034383</v>
+        <v>648.04446103438295</v>
       </c>
       <c r="E37" s="38">
         <f t="shared" si="14"/>
-        <v>518.290592438013</v>
+        <v>518.29059243801305</v>
       </c>
       <c r="F37" s="38">
         <f t="shared" si="14"/>
@@ -5423,7 +4901,7 @@
       </c>
       <c r="G37" s="38">
         <f t="shared" si="14"/>
-        <v>22.6815561362034</v>
+        <v>22.681556136203401</v>
       </c>
       <c r="H37" s="38">
         <f t="shared" si="14"/>
@@ -5431,29 +4909,29 @@
       </c>
       <c r="I37" s="9">
         <f t="shared" si="14"/>
-        <v>2.77777777777778</v>
+        <v>2.7777777777777799</v>
       </c>
       <c r="J37" s="9">
         <f t="shared" si="14"/>
-        <v>2.22222222222222</v>
+        <v>2.2222222222222201</v>
       </c>
       <c r="K37" s="9">
         <f t="shared" si="14"/>
-        <v>1.66666666666667</v>
+        <v>1.6666666666666701</v>
       </c>
       <c r="L37" s="9">
         <f t="shared" si="14"/>
-        <v>1.38888888888889</v>
+        <v>1.3888888888888899</v>
       </c>
       <c r="M37" s="9">
         <f t="shared" si="14"/>
-        <v>1.13888888888889</v>
+        <v>1.1388888888888899</v>
       </c>
       <c r="N37" s="9">
         <f t="shared" si="14"/>
         <v>0.3</v>
       </c>
-      <c r="O37" s="180" t="s">
+      <c r="O37" s="175" t="s">
         <v>70</v>
       </c>
       <c r="S37" t="str">
@@ -5484,11 +4962,11 @@
     <row r="38" spans="1:25">
       <c r="C38" s="38">
         <f t="shared" ref="C38:N38" si="15">C22</f>
-        <v>1259.79843225084</v>
+        <v>1259.7984322508401</v>
       </c>
       <c r="D38" s="38">
         <f t="shared" si="15"/>
-        <v>894.301356227448</v>
+        <v>894.30135622744797</v>
       </c>
       <c r="E38" s="38">
         <f t="shared" si="15"/>
@@ -5496,15 +4974,15 @@
       </c>
       <c r="F38" s="38">
         <f t="shared" si="15"/>
-        <v>44.0929451287794</v>
+        <v>44.092945128779398</v>
       </c>
       <c r="G38" s="38">
         <f t="shared" si="15"/>
-        <v>31.3005474679607</v>
+        <v>31.300547467960701</v>
       </c>
       <c r="H38" s="38">
         <f t="shared" si="15"/>
-        <v>17.325</v>
+        <v>17.324999999999999</v>
       </c>
       <c r="I38" s="9">
         <f t="shared" si="15"/>
@@ -5530,7 +5008,7 @@
         <f t="shared" si="15"/>
         <v>0.3</v>
       </c>
-      <c r="O38" s="180" t="s">
+      <c r="O38" s="175" t="s">
         <v>70</v>
       </c>
       <c r="S38" t="str">
@@ -5559,77 +5037,77 @@
       </c>
     </row>
     <row r="39" spans="1:25">
-      <c r="A39" s="182" t="str">
+      <c r="A39" s="177" t="str">
         <f>A35</f>
         <v>HH2</v>
       </c>
-      <c r="B39" s="182" t="s">
+      <c r="B39" s="177" t="s">
         <v>69</v>
       </c>
-      <c r="C39" s="183">
+      <c r="C39" s="178">
         <f>C29</f>
         <v>900</v>
       </c>
-      <c r="D39" s="183">
+      <c r="D39" s="178">
         <f t="shared" ref="D39:H39" si="16">D29</f>
         <v>850</v>
       </c>
-      <c r="E39" s="183">
+      <c r="E39" s="178">
         <f t="shared" si="16"/>
         <v>800</v>
       </c>
-      <c r="F39" s="183">
+      <c r="F39" s="178">
         <f t="shared" si="16"/>
         <v>36</v>
       </c>
-      <c r="G39" s="183">
+      <c r="G39" s="178">
         <f t="shared" si="16"/>
         <v>34</v>
       </c>
-      <c r="H39" s="183">
+      <c r="H39" s="178">
         <f t="shared" si="16"/>
         <v>32</v>
       </c>
-      <c r="I39" s="184">
+      <c r="I39" s="179">
         <v>1.25</v>
       </c>
-      <c r="J39" s="184">
+      <c r="J39" s="179">
         <v>0.12</v>
       </c>
-      <c r="K39" s="184">
+      <c r="K39" s="179">
         <v>1.25</v>
       </c>
-      <c r="L39" s="184">
+      <c r="L39" s="179">
         <v>0.12</v>
       </c>
-      <c r="M39" s="184">
+      <c r="M39" s="179">
         <v>1.25</v>
       </c>
-      <c r="N39" s="184">
+      <c r="N39" s="179">
         <v>0.12</v>
       </c>
-      <c r="O39" s="182" t="s">
+      <c r="O39" s="177" t="s">
         <v>77</v>
       </c>
-      <c r="P39" s="182">
+      <c r="P39" s="177">
         <v>25</v>
       </c>
-      <c r="Q39" s="182">
-        <v>31.536</v>
-      </c>
-      <c r="R39" s="182"/>
-      <c r="S39" s="182" t="str">
+      <c r="Q39" s="177">
+        <v>31.536000000000001</v>
+      </c>
+      <c r="R39" s="177"/>
+      <c r="S39" s="177" t="str">
         <f t="shared" si="5"/>
         <v>PRE</v>
       </c>
-      <c r="T39" s="182" t="str">
+      <c r="T39" s="177" t="str">
         <f t="shared" si="6"/>
         <v>H2prd_Gas_ATR_CCS</v>
       </c>
-      <c r="U39" s="182" t="s">
+      <c r="U39" s="177" t="s">
         <v>78</v>
       </c>
-      <c r="V39" s="182" t="s">
+      <c r="V39" s="177" t="s">
         <v>71</v>
       </c>
       <c r="W39" t="s">
@@ -5650,39 +5128,37 @@
     <mergeCell ref="O1:O4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
-  <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B3:Q12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="9" style="52"/>
-    <col min="2" max="2" width="12.8636363636364" style="52" customWidth="1"/>
-    <col min="3" max="3" width="8.86363636363636" style="52" customWidth="1"/>
-    <col min="4" max="4" width="14.8636363636364" style="52" customWidth="1"/>
+    <col min="2" max="2" width="12.86328125" style="52" customWidth="1"/>
+    <col min="3" max="3" width="8.86328125" style="52" customWidth="1"/>
+    <col min="4" max="4" width="14.86328125" style="52" customWidth="1"/>
     <col min="5" max="5" width="9" style="52" customWidth="1"/>
-    <col min="6" max="6" width="10.2636363636364" style="52" customWidth="1"/>
-    <col min="7" max="7" width="4.6" style="52" customWidth="1"/>
-    <col min="8" max="8" width="11.6" style="52" customWidth="1"/>
-    <col min="9" max="9" width="11.2636363636364" style="52" customWidth="1"/>
-    <col min="10" max="10" width="11.4" style="52" customWidth="1"/>
-    <col min="11" max="11" width="5.6" style="52" customWidth="1"/>
+    <col min="6" max="6" width="10.265625" style="52" customWidth="1"/>
+    <col min="7" max="7" width="4.59765625" style="52" customWidth="1"/>
+    <col min="8" max="8" width="11.59765625" style="52" customWidth="1"/>
+    <col min="9" max="9" width="11.265625" style="52" customWidth="1"/>
+    <col min="10" max="10" width="11.3984375" style="52" customWidth="1"/>
+    <col min="11" max="11" width="5.59765625" style="52" customWidth="1"/>
     <col min="12" max="12" width="9" style="52"/>
-    <col min="13" max="13" width="11.2636363636364" style="52" customWidth="1"/>
-    <col min="14" max="14" width="12.8636363636364" style="52" customWidth="1"/>
-    <col min="15" max="15" width="15.2636363636364" style="52" customWidth="1"/>
-    <col min="16" max="16" width="4.6" style="52" customWidth="1"/>
+    <col min="13" max="13" width="11.265625" style="52" customWidth="1"/>
+    <col min="14" max="14" width="12.86328125" style="52" customWidth="1"/>
+    <col min="15" max="15" width="15.265625" style="52" customWidth="1"/>
+    <col min="16" max="16" width="4.59765625" style="52" customWidth="1"/>
     <col min="17" max="17" width="5" style="52" customWidth="1"/>
     <col min="18" max="16384" width="9" style="52"/>
   </cols>
   <sheetData>
-    <row r="3" ht="17.75" spans="2:17">
+    <row r="3" spans="2:17" ht="16.899999999999999">
       <c r="D3" s="53" t="s">
         <v>79</v>
       </c>
@@ -5694,7 +5170,7 @@
       <c r="P3" s="54"/>
       <c r="Q3" s="54"/>
     </row>
-    <row r="4" ht="16" spans="2:17">
+    <row r="4" spans="2:17" ht="14.25">
       <c r="B4" s="55" t="s">
         <v>80</v>
       </c>
@@ -5752,7 +5228,7 @@
         <v>91</v>
       </c>
       <c r="E5" s="52">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="F5" s="56">
         <v>0.6</v>
@@ -5761,10 +5237,10 @@
         <v>0.6</v>
       </c>
       <c r="H5" s="56">
-        <v>189.216</v>
+        <v>189.21600000000001</v>
       </c>
       <c r="I5" s="56">
-        <v>88.3008</v>
+        <v>88.300799999999995</v>
       </c>
       <c r="J5" s="52">
         <v>60</v>
@@ -5801,7 +5277,7 @@
         <v>91</v>
       </c>
       <c r="E6" s="52">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="F6" s="56">
         <v>0.6</v>
@@ -5810,10 +5286,10 @@
         <v>0.6</v>
       </c>
       <c r="H6" s="56">
-        <v>189.216</v>
+        <v>189.21600000000001</v>
       </c>
       <c r="I6" s="56">
-        <v>88.3008</v>
+        <v>88.300799999999995</v>
       </c>
       <c r="J6" s="52">
         <v>60</v>
@@ -5847,7 +5323,7 @@
         <v>91</v>
       </c>
       <c r="E7" s="52">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="F7" s="56">
         <v>0.1</v>
@@ -5856,16 +5332,16 @@
         <v>0.6</v>
       </c>
       <c r="H7" s="56">
-        <v>141.912</v>
+        <v>141.91200000000001</v>
       </c>
       <c r="I7" s="56">
-        <v>75.6864</v>
+        <v>75.686400000000006</v>
       </c>
       <c r="J7" s="52">
         <v>60</v>
       </c>
       <c r="K7" s="57">
-        <v>0.869565217391304</v>
+        <v>0.86956521739130399</v>
       </c>
       <c r="N7" s="52" t="str">
         <f t="shared" si="0"/>
@@ -5893,7 +5369,7 @@
         <v>91</v>
       </c>
       <c r="E8" s="52">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="F8" s="56">
         <v>0.3</v>
@@ -5928,7 +5404,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="9" ht="13" spans="2:17">
+    <row r="9" spans="2:17" ht="13.15">
       <c r="B9" s="58" t="s">
         <v>99</v>
       </c>
@@ -5940,7 +5416,7 @@
       </c>
       <c r="E9" s="52">
         <f t="shared" ref="E9:K9" si="1">E7</f>
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="F9" s="56">
         <f t="shared" si="1"/>
@@ -5952,11 +5428,11 @@
       </c>
       <c r="H9" s="56">
         <f t="shared" si="1"/>
-        <v>141.912</v>
+        <v>141.91200000000001</v>
       </c>
       <c r="I9" s="56">
         <f t="shared" si="1"/>
-        <v>75.6864</v>
+        <v>75.686400000000006</v>
       </c>
       <c r="J9" s="52">
         <f t="shared" si="1"/>
@@ -5964,7 +5440,7 @@
       </c>
       <c r="K9" s="57">
         <f t="shared" si="1"/>
-        <v>0.869565217391304</v>
+        <v>0.86956521739130399</v>
       </c>
       <c r="N9" s="52" t="str">
         <f t="shared" si="0"/>
@@ -5993,7 +5469,7 @@
       </c>
       <c r="E10" s="52">
         <f>E8</f>
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="F10" s="56"/>
       <c r="G10" s="56"/>
@@ -6062,34 +5538,33 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:AK40"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="8" max="8" width="17.6" customWidth="1"/>
-    <col min="10" max="10" width="10.8636363636364" customWidth="1"/>
+    <col min="8" max="8" width="17.59765625" customWidth="1"/>
+    <col min="10" max="10" width="10.86328125" customWidth="1"/>
     <col min="11" max="13" width="5" customWidth="1"/>
-    <col min="14" max="14" width="8.4" customWidth="1"/>
+    <col min="14" max="14" width="8.3984375" customWidth="1"/>
     <col min="15" max="15" width="2" customWidth="1"/>
-    <col min="16" max="16" width="3.6" customWidth="1"/>
-    <col min="17" max="17" width="17.6" customWidth="1"/>
+    <col min="16" max="16" width="3.59765625" customWidth="1"/>
+    <col min="17" max="17" width="17.59765625" customWidth="1"/>
     <col min="21" max="21" width="2" customWidth="1"/>
-    <col min="22" max="22" width="17.6" customWidth="1"/>
+    <col min="22" max="22" width="17.59765625" customWidth="1"/>
     <col min="23" max="25" width="6" customWidth="1"/>
     <col min="26" max="26" width="2" customWidth="1"/>
-    <col min="27" max="27" width="17.6" customWidth="1"/>
-    <col min="28" max="28" width="11.4" customWidth="1"/>
+    <col min="27" max="27" width="17.59765625" customWidth="1"/>
+    <col min="28" max="28" width="11.3984375" customWidth="1"/>
     <col min="29" max="31" width="5" customWidth="1"/>
-    <col min="33" max="33" width="19.8636363636364" customWidth="1"/>
-    <col min="34" max="34" width="5.6" customWidth="1"/>
+    <col min="33" max="33" width="19.86328125" customWidth="1"/>
+    <col min="34" max="34" width="5.59765625" customWidth="1"/>
     <col min="35" max="37" width="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6253,7 +5728,7 @@
         <v>439.05</v>
       </c>
       <c r="N3" s="39">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="O3" s="38"/>
       <c r="P3" s="40">
@@ -6265,15 +5740,15 @@
       </c>
       <c r="R3" s="39">
         <f>$P3*K3</f>
-        <v>29.109</v>
+        <v>29.109000000000002</v>
       </c>
       <c r="S3" s="39">
         <f t="shared" ref="S3:T5" si="2">$P3*L3</f>
-        <v>13.226</v>
+        <v>13.226000000000001</v>
       </c>
       <c r="T3" s="39">
         <f t="shared" si="2"/>
-        <v>8.781</v>
+        <v>8.7810000000000006</v>
       </c>
       <c r="V3" t="str">
         <f t="shared" ref="V3:V5" si="3">$H3</f>
@@ -6324,7 +5799,7 @@
         <v>661.3</v>
       </c>
       <c r="E4" s="37">
-        <v>138.45</v>
+        <v>138.44999999999999</v>
       </c>
       <c r="F4" s="37">
         <v>1368.75</v>
@@ -6342,17 +5817,17 @@
         <v>338.75</v>
       </c>
       <c r="L4" s="38">
-        <v>138.45</v>
+        <v>138.44999999999999</v>
       </c>
       <c r="M4" s="38">
         <v>87.3</v>
       </c>
       <c r="N4" s="39">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="O4" s="39"/>
       <c r="P4" s="40">
-        <v>0.035</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="Q4" t="str">
         <f t="shared" si="1"/>
@@ -6360,28 +5835,28 @@
       </c>
       <c r="R4" s="39">
         <f t="shared" ref="R4:R5" si="4">$P4*K4</f>
-        <v>11.85625</v>
+        <v>11.856249999999999</v>
       </c>
       <c r="S4" s="39">
         <f t="shared" si="2"/>
-        <v>4.84575</v>
+        <v>4.8457499999999998</v>
       </c>
       <c r="T4" s="39">
         <f t="shared" si="2"/>
-        <v>3.0555</v>
+        <v>3.0554999999999999</v>
       </c>
       <c r="V4" t="str">
         <f t="shared" si="3"/>
         <v>H2Conv_LOHC</v>
       </c>
       <c r="W4">
-        <v>0.925</v>
+        <v>0.92500000000000004</v>
       </c>
       <c r="X4">
         <v>0.95</v>
       </c>
       <c r="Y4">
-        <v>0.975</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="AA4" t="str">
         <f t="shared" ref="AA4:AA5" si="5">H4</f>
@@ -6443,7 +5918,7 @@
         <v>799.5</v>
       </c>
       <c r="N5" s="39">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="O5" s="39"/>
       <c r="P5" s="40">
@@ -6489,7 +5964,7 @@
         <v>0.255</v>
       </c>
       <c r="AD5" s="9">
-        <v>0.225</v>
+        <v>0.22500000000000001</v>
       </c>
       <c r="AE5" s="9">
         <v>0.1875</v>
@@ -6516,7 +5991,7 @@
         <v>0.02</v>
       </c>
       <c r="E6" s="44">
-        <v>0.035</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="F6" s="44">
         <v>0.04</v>
@@ -6536,7 +6011,7 @@
         <v>0.875</v>
       </c>
       <c r="E7" s="44">
-        <v>0.925</v>
+        <v>0.92500000000000004</v>
       </c>
       <c r="F7" s="44">
         <v>0.95</v>
@@ -6579,7 +6054,7 @@
         <v>0.875</v>
       </c>
       <c r="E9" s="44">
-        <v>0.975</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="F9" s="44">
         <v>1</v>
@@ -6590,7 +6065,7 @@
       </c>
       <c r="I9">
         <f>F11*3.6/120</f>
-        <v>0.225</v>
+        <v>0.22500000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:37">
@@ -6764,7 +6239,7 @@
         <v>752.1</v>
       </c>
       <c r="F14" s="48">
-        <v>649.45</v>
+        <v>649.45000000000005</v>
       </c>
       <c r="H14" t="s">
         <v>143</v>
@@ -6785,11 +6260,11 @@
         <v>276.55</v>
       </c>
       <c r="N14" s="39">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="O14" s="38"/>
       <c r="P14" s="40">
-        <v>0.035</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="Q14" t="str">
         <f t="shared" ref="Q14:Q16" si="6">$H14</f>
@@ -6797,15 +6272,15 @@
       </c>
       <c r="R14" s="39">
         <f>$P14*K14</f>
-        <v>40.39175</v>
+        <v>40.391750000000002</v>
       </c>
       <c r="S14" s="39">
         <f t="shared" ref="S14:T16" si="7">$P14*L14</f>
-        <v>16.02475</v>
+        <v>16.024750000000001</v>
       </c>
       <c r="T14" s="39">
         <f t="shared" si="7"/>
-        <v>9.67925</v>
+        <v>9.6792499999999997</v>
       </c>
       <c r="V14" t="str">
         <f t="shared" ref="V14:V16" si="8">$H14</f>
@@ -6825,10 +6300,10 @@
         <v>0.06</v>
       </c>
       <c r="AD14" s="9">
-        <v>0.045</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="AE14" s="9">
-        <v>0.0225</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="AF14" s="9">
         <v>0.4</v>
@@ -6874,11 +6349,11 @@
         <v>169.75</v>
       </c>
       <c r="N15" s="39">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="O15" s="39"/>
       <c r="P15" s="40">
-        <v>0.045</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="Q15" t="str">
         <f t="shared" si="6"/>
@@ -6886,15 +6361,15 @@
       </c>
       <c r="R15" s="39">
         <f t="shared" ref="R15:R16" si="9">$P15*K15</f>
-        <v>33.8445</v>
+        <v>33.844499999999996</v>
       </c>
       <c r="S15" s="39">
         <f t="shared" si="7"/>
-        <v>14.4675</v>
+        <v>14.467499999999999</v>
       </c>
       <c r="T15" s="39">
         <f t="shared" si="7"/>
-        <v>7.63875</v>
+        <v>7.6387499999999999</v>
       </c>
       <c r="V15" t="str">
         <f t="shared" si="8"/>
@@ -6954,7 +6429,7 @@
         <v>16</v>
       </c>
       <c r="K16" s="38">
-        <v>649.45</v>
+        <v>649.45000000000005</v>
       </c>
       <c r="L16" s="38">
         <v>267.3</v>
@@ -6963,11 +6438,11 @@
         <v>125.45</v>
       </c>
       <c r="N16" s="39">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
       <c r="O16" s="39"/>
       <c r="P16" s="40">
-        <v>0.035</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="Q16" t="str">
         <f t="shared" si="6"/>
@@ -6979,11 +6454,11 @@
       </c>
       <c r="S16" s="39">
         <f t="shared" si="7"/>
-        <v>9.3555</v>
+        <v>9.3554999999999993</v>
       </c>
       <c r="T16" s="39">
         <f t="shared" si="7"/>
-        <v>4.39075</v>
+        <v>4.3907499999999997</v>
       </c>
       <c r="V16" t="str">
         <f t="shared" si="8"/>
@@ -7000,13 +6475,13 @@
         <v>102</v>
       </c>
       <c r="AC16" s="9">
-        <v>0.0225</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="AD16" s="9">
-        <v>0.01575</v>
+        <v>1.575E-2</v>
       </c>
       <c r="AE16" s="9">
-        <v>0.009</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="AF16" s="9">
         <v>0.4</v>
@@ -7030,13 +6505,13 @@
       </c>
       <c r="C17" s="49"/>
       <c r="D17" s="44">
-        <v>0.035</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="E17" s="44">
-        <v>0.045</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="F17" s="44">
-        <v>0.035</v>
+        <v>3.5000000000000003E-2</v>
       </c>
     </row>
     <row r="18" spans="1:33">
@@ -7092,7 +6567,7 @@
       </c>
       <c r="J19" s="39">
         <f t="shared" si="11"/>
-        <v>0.0225</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="AA19" t="s">
         <v>120</v>
@@ -7129,11 +6604,11 @@
         <v>2</v>
       </c>
       <c r="F20" s="37">
-        <v>0.525</v>
+        <v>0.52500000000000002</v>
       </c>
       <c r="H20" s="39">
         <f t="shared" ref="H20:H24" si="12">D20*3.6/120</f>
-        <v>0.045</v>
+        <v>4.4999999999999998E-2</v>
       </c>
       <c r="I20" s="39">
         <f t="shared" si="11"/>
@@ -7141,7 +6616,7 @@
       </c>
       <c r="J20" s="39">
         <f t="shared" si="11"/>
-        <v>0.01575</v>
+        <v>1.575E-2</v>
       </c>
       <c r="AA20" t="str">
         <f>V14</f>
@@ -7154,10 +6629,10 @@
         <v>0.42</v>
       </c>
       <c r="AD20" s="9">
-        <v>0.3315</v>
+        <v>0.33150000000000002</v>
       </c>
       <c r="AE20" s="9">
-        <v>0.243</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="AF20" t="s">
         <v>149</v>
@@ -7183,7 +6658,7 @@
       </c>
       <c r="H21" s="39">
         <f t="shared" si="12"/>
-        <v>0.0225</v>
+        <v>2.2499999999999999E-2</v>
       </c>
       <c r="I21" s="39">
         <f t="shared" si="11"/>
@@ -7191,7 +6666,7 @@
       </c>
       <c r="J21" s="39">
         <f t="shared" si="11"/>
-        <v>0.009</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="AA21" t="str">
         <f>V15</f>
@@ -7204,10 +6679,10 @@
         <v>0.51</v>
       </c>
       <c r="AD21" s="9">
-        <v>0.4245</v>
+        <v>0.42449999999999999</v>
       </c>
       <c r="AE21" s="9">
-        <v>0.339</v>
+        <v>0.33900000000000002</v>
       </c>
       <c r="AF21" t="s">
         <v>149</v>
@@ -7265,11 +6740,11 @@
       </c>
       <c r="H23" s="39">
         <f t="shared" si="12"/>
-        <v>0.3315</v>
+        <v>0.33150000000000002</v>
       </c>
       <c r="I23" s="39">
         <f t="shared" si="11"/>
-        <v>0.4245</v>
+        <v>0.42449999999999999</v>
       </c>
       <c r="J23" s="39">
         <f t="shared" si="11"/>
@@ -7293,11 +6768,11 @@
       </c>
       <c r="H24" s="39">
         <f t="shared" si="12"/>
-        <v>0.243</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="I24" s="39">
         <f t="shared" si="11"/>
-        <v>0.339</v>
+        <v>0.33900000000000002</v>
       </c>
       <c r="J24" s="39">
         <f t="shared" si="11"/>
@@ -7463,37 +6938,35 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B3:Y5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="11.2636363636364" customWidth="1"/>
-    <col min="3" max="3" width="14.6" customWidth="1"/>
-    <col min="4" max="4" width="26.4" customWidth="1"/>
-    <col min="5" max="5" width="20.2636363636364" customWidth="1"/>
+    <col min="2" max="2" width="11.265625" customWidth="1"/>
+    <col min="3" max="3" width="14.59765625" customWidth="1"/>
+    <col min="4" max="4" width="26.3984375" customWidth="1"/>
+    <col min="5" max="5" width="20.265625" customWidth="1"/>
     <col min="6" max="6" width="5" customWidth="1"/>
-    <col min="7" max="7" width="4.6" customWidth="1"/>
+    <col min="7" max="7" width="4.59765625" customWidth="1"/>
     <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="10.2636363636364" customWidth="1"/>
-    <col min="10" max="10" width="7.86363636363636" customWidth="1"/>
-    <col min="12" max="12" width="17.8636363636364" customWidth="1"/>
-    <col min="13" max="13" width="9.4" customWidth="1"/>
+    <col min="9" max="9" width="10.265625" customWidth="1"/>
+    <col min="10" max="10" width="7.86328125" customWidth="1"/>
+    <col min="12" max="12" width="17.86328125" customWidth="1"/>
+    <col min="13" max="13" width="9.3984375" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="8.86363636363636" customWidth="1"/>
+    <col min="15" max="15" width="8.86328125" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="6.86363636363636" customWidth="1"/>
-    <col min="18" max="18" width="11.8636363636364" customWidth="1"/>
-    <col min="19" max="19" width="7.86363636363636" customWidth="1"/>
-    <col min="20" max="20" width="12.8636363636364" customWidth="1"/>
-    <col min="21" max="21" width="4.6" customWidth="1"/>
+    <col min="17" max="17" width="6.86328125" customWidth="1"/>
+    <col min="18" max="18" width="11.86328125" customWidth="1"/>
+    <col min="19" max="19" width="7.86328125" customWidth="1"/>
+    <col min="20" max="20" width="12.86328125" customWidth="1"/>
+    <col min="21" max="21" width="4.59765625" customWidth="1"/>
     <col min="22" max="22" width="9" customWidth="1"/>
-    <col min="23" max="23" width="4.4" customWidth="1"/>
+    <col min="23" max="23" width="4.3984375" customWidth="1"/>
     <col min="24" max="24" width="5" customWidth="1"/>
     <col min="25" max="25" width="9" customWidth="1"/>
   </cols>
@@ -7619,16 +7092,16 @@
         <v>71</v>
       </c>
       <c r="S5" s="9">
-        <v>2.13470319634703</v>
+        <v>2.1347031963470302</v>
       </c>
       <c r="T5" s="9">
         <v>1.72231735159817</v>
       </c>
       <c r="U5" s="9">
-        <v>0.5525</v>
+        <v>0.55249999999999999</v>
       </c>
       <c r="V5" s="9">
-        <v>0.5525</v>
+        <v>0.55249999999999999</v>
       </c>
       <c r="W5">
         <v>20</v>
@@ -7637,49 +7110,49 @@
         <v>0.85</v>
       </c>
       <c r="Y5">
-        <v>31.536</v>
+        <v>31.536000000000001</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="B1:BP66"/>
-  <sheetFormatPr defaultColWidth="8.8" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="32.5272727272727" customWidth="1"/>
-    <col min="3" max="3" width="30.7272727272727" customWidth="1"/>
+    <col min="2" max="2" width="32.53125" customWidth="1"/>
+    <col min="3" max="3" width="30.73046875" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
-    <col min="5" max="5" width="29.9272727272727" customWidth="1"/>
-    <col min="6" max="9" width="33.7272727272727" customWidth="1"/>
-    <col min="10" max="10" width="19.2636363636364" customWidth="1"/>
-    <col min="11" max="11" width="14.6" customWidth="1"/>
-    <col min="12" max="12" width="14.2636363636364" customWidth="1"/>
-    <col min="13" max="13" width="13.0636363636364" customWidth="1"/>
-    <col min="14" max="14" width="12.8" customWidth="1"/>
-    <col min="15" max="15" width="6.8" customWidth="1"/>
-    <col min="16" max="16" width="15.3363636363636" customWidth="1"/>
-    <col min="17" max="17" width="6.2" customWidth="1"/>
-    <col min="18" max="18" width="14.5272727272727" customWidth="1"/>
-    <col min="23" max="23" width="20.2" customWidth="1"/>
-    <col min="24" max="24" width="18.5272727272727" customWidth="1"/>
-    <col min="25" max="25" width="19.2" customWidth="1"/>
-    <col min="32" max="32" width="21.2636363636364" customWidth="1"/>
-    <col min="36" max="36" width="13.5272727272727" customWidth="1"/>
-    <col min="40" max="40" width="19.6363636363636" customWidth="1"/>
-    <col min="43" max="43" width="13.0909090909091" customWidth="1"/>
-    <col min="44" max="44" width="7.09090909090909" customWidth="1"/>
-    <col min="46" max="46" width="15.3636363636364" customWidth="1"/>
-    <col min="48" max="48" width="13.2" customWidth="1"/>
-    <col min="49" max="49" width="5.26363636363636" customWidth="1"/>
-    <col min="50" max="50" width="5.92727272727273" customWidth="1"/>
+    <col min="5" max="5" width="29.9296875" customWidth="1"/>
+    <col min="6" max="9" width="33.73046875" customWidth="1"/>
+    <col min="10" max="10" width="19.265625" customWidth="1"/>
+    <col min="11" max="11" width="14.59765625" customWidth="1"/>
+    <col min="12" max="12" width="14.265625" customWidth="1"/>
+    <col min="13" max="13" width="13.06640625" customWidth="1"/>
+    <col min="14" max="14" width="12.796875" customWidth="1"/>
+    <col min="15" max="15" width="6.796875" customWidth="1"/>
+    <col min="16" max="16" width="15.33203125" customWidth="1"/>
+    <col min="17" max="17" width="6.19921875" customWidth="1"/>
+    <col min="18" max="18" width="14.53125" customWidth="1"/>
+    <col min="23" max="23" width="20.19921875" customWidth="1"/>
+    <col min="24" max="24" width="18.53125" customWidth="1"/>
+    <col min="25" max="25" width="19.19921875" customWidth="1"/>
+    <col min="32" max="32" width="21.265625" customWidth="1"/>
+    <col min="36" max="36" width="13.53125" customWidth="1"/>
+    <col min="40" max="40" width="19.59765625" customWidth="1"/>
+    <col min="41" max="41" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="13.06640625" customWidth="1"/>
+    <col min="44" max="44" width="7.06640625" customWidth="1"/>
+    <col min="46" max="46" width="15.33203125" customWidth="1"/>
+    <col min="48" max="48" width="13.19921875" customWidth="1"/>
+    <col min="49" max="49" width="5.265625" customWidth="1"/>
+    <col min="50" max="50" width="5.9296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:53">
@@ -7787,7 +7260,7 @@
         <v>185</v>
       </c>
       <c r="Z4" s="3">
-        <v>0.095</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="AA4" s="3">
         <v>0</v>
@@ -7802,7 +7275,7 @@
         <v>3.528</v>
       </c>
       <c r="AE4" s="3">
-        <v>0.946</v>
+        <v>0.94599999999999995</v>
       </c>
       <c r="AF4" s="3">
         <v>1.085</v>
@@ -8193,7 +7666,7 @@
         <v>0.92</v>
       </c>
       <c r="I16" s="9">
-        <v>1.314</v>
+        <v>1.3140000000000001</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -8232,7 +7705,7 @@
         <v>0.9</v>
       </c>
       <c r="AM16" s="9">
-        <v>1.314</v>
+        <v>1.3140000000000001</v>
       </c>
       <c r="AN16">
         <v>1</v>
@@ -8253,7 +7726,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="16" spans="2:68">
+    <row r="17" spans="2:68" s="1" customFormat="1" ht="15.4">
       <c r="D17" s="11"/>
       <c r="F17" s="1" t="s">
         <v>212</v>
@@ -8265,7 +7738,7 @@
       <c r="I17" s="12"/>
       <c r="K17" s="12">
         <f>1/H16</f>
-        <v>1.08695652173913</v>
+        <v>1.0869565217391299</v>
       </c>
       <c r="W17"/>
       <c r="Y17" s="13" t="s">
@@ -8291,7 +7764,7 @@
       <c r="AM17" s="9"/>
       <c r="AN17"/>
       <c r="AO17" s="9">
-        <v>1.08695652173913</v>
+        <v>1</v>
       </c>
       <c r="AQ17"/>
       <c r="AR17"/>
@@ -8353,7 +7826,7 @@
         <v>215</v>
       </c>
       <c r="I19" s="9">
-        <v>29.89194313</v>
+        <v>29.891943130000001</v>
       </c>
       <c r="L19">
         <v>1</v>
@@ -8382,7 +7855,7 @@
       </c>
       <c r="AM19" s="9">
         <f>AM16</f>
-        <v>1.314</v>
+        <v>1.3140000000000001</v>
       </c>
       <c r="AN19">
         <v>1</v>
@@ -8413,7 +7886,7 @@
       </c>
       <c r="AM20" s="9"/>
       <c r="AO20" s="9">
-        <v>1.08695652173913</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="2:68">
@@ -8450,7 +7923,7 @@
       </c>
       <c r="AM22" s="9">
         <f>AM19</f>
-        <v>1.314</v>
+        <v>1.3140000000000001</v>
       </c>
       <c r="AN22">
         <v>1</v>
@@ -8495,7 +7968,7 @@
       <c r="AL23" s="10"/>
       <c r="AM23" s="9"/>
       <c r="AO23" s="9">
-        <v>1.08695652173913</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="2:68">
@@ -8577,7 +8050,7 @@
       </c>
       <c r="AM25" s="9">
         <f>AM22</f>
-        <v>1.314</v>
+        <v>1.3140000000000001</v>
       </c>
       <c r="AN25">
         <v>1</v>
@@ -8625,7 +8098,7 @@
       <c r="AL26" s="10"/>
       <c r="AM26" s="9"/>
       <c r="AO26" s="9">
-        <v>1.08695652173913</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="2:68">
@@ -8666,7 +8139,7 @@
       </c>
       <c r="AM28" s="9">
         <f>AM25</f>
-        <v>1.314</v>
+        <v>1.3140000000000001</v>
       </c>
       <c r="AN28">
         <v>1</v>
@@ -8705,7 +8178,7 @@
       <c r="AL29" s="10"/>
       <c r="AM29" s="9"/>
       <c r="AO29" s="9">
-        <v>1.08695652173913</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="2:68">
@@ -8756,7 +8229,7 @@
       </c>
       <c r="AM31" s="9">
         <f>AM28</f>
-        <v>1.314</v>
+        <v>1.3140000000000001</v>
       </c>
       <c r="AN31">
         <v>1</v>
@@ -8799,7 +8272,7 @@
       </c>
       <c r="AM32" s="9"/>
       <c r="AO32" s="9">
-        <v>1.08695652173913</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="2:51">
@@ -8814,7 +8287,7 @@
       </c>
       <c r="E33" s="20">
         <f>[6]EnergyUseFromEverBatt_Min_!$AW$6</f>
-        <v>0.0473</v>
+        <v>4.7300000000000002E-2</v>
       </c>
       <c r="AH33" s="5"/>
       <c r="AJ33" s="5" t="s">
@@ -8828,7 +8301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" ht="16" spans="2:51">
+    <row r="34" spans="2:51" ht="15.4">
       <c r="B34" s="6" t="s">
         <v>188</v>
       </c>
@@ -8841,7 +8314,7 @@
       </c>
       <c r="E34" s="20">
         <f>[6]EnergyUseFromEverBatt_Min_!$AW$7</f>
-        <v>0.171166666666667</v>
+        <v>0.17116666666666699</v>
       </c>
       <c r="AF34" t="s">
         <v>199</v>
@@ -8885,7 +8358,7 @@
         <v>1566.7</v>
       </c>
     </row>
-    <row r="35" ht="16" spans="2:51">
+    <row r="35" spans="2:51" ht="15.4">
       <c r="B35" s="6" t="s">
         <v>188</v>
       </c>
@@ -8898,7 +8371,7 @@
       </c>
       <c r="E35" s="20">
         <f>[6]EnergyUseFromEverBatt_Min_!$AW$8</f>
-        <v>0.466366666666667</v>
+        <v>0.46636666666666698</v>
       </c>
       <c r="AJ35" t="s">
         <v>212</v>
@@ -8907,10 +8380,10 @@
         <v>212</v>
       </c>
       <c r="AO35">
-        <v>1.09</v>
-      </c>
-    </row>
-    <row r="36" ht="16" spans="2:51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:51" ht="15.4">
       <c r="B36" s="6" t="s">
         <v>188</v>
       </c>
@@ -8923,7 +8396,7 @@
       </c>
       <c r="E36" s="20">
         <f>[6]EnergyUseFromEverBatt_Min_!$AW$9</f>
-        <v>0.0956666666666667</v>
+        <v>9.5666666666666705E-2</v>
       </c>
       <c r="AJ36" s="5" t="s">
         <v>214</v>
@@ -8960,7 +8433,7 @@
       <c r="R43" s="8"/>
       <c r="S43" s="15"/>
     </row>
-    <row r="44" ht="16" spans="2:51">
+    <row r="44" spans="2:51" ht="15.4">
       <c r="B44" s="22" t="s">
         <v>80</v>
       </c>
@@ -8996,7 +8469,7 @@
       <c r="R44" s="8"/>
       <c r="S44" s="8"/>
     </row>
-    <row r="45" ht="16" spans="2:51">
+    <row r="45" spans="2:51" ht="15.4">
       <c r="B45" s="27" t="s">
         <v>185</v>
       </c>
@@ -9368,7 +8841,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
-  <legacyDrawing r:id="rId2"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>